<commit_message>
Committing Generated Files 40
</commit_message>
<xml_diff>
--- a/manual_tests/login_approved_manual_tests.xlsx
+++ b/manual_tests/login_approved_manual_tests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -470,7 +470,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Verify login page loads and UI elements are visible</t>
+          <t>Verify login page UI elements are visible</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -486,19 +486,18 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Open the login page URL http://172.21.166.115/washtabui/login?data=undefined
-Observe the login page interface
-Verify User Name textbox is visible
-Verify Password field is visible
-Verify characters entered into Password field are masked
-Verify SIGN IN button is visible
-Verify Home control is visible
-Verify Arrow Back control is visible</t>
+          <t>Navigate to http://172.21.166.115/washtabui/login?data=undefined
+Verify the browser URL matches the login page URL
+Check presence of username_textbox
+Check presence of password_textbox
+Check presence of sign_in_button
+Check presence of back_navigation_button
+Check presence of home_navigation_button</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Login page loads without error and displays User Name textbox, Password masked input field, SIGN IN button, Home control, and Arrow Back control. The browser URL remains http://172.21.166.115/washtabui/login?data=undefined.</t>
+          <t>Login page loads successfully at the specified URL and the username_textbox, password_textbox, SIGN IN button, back_navigation_button, and home_navigation_button are visible and interactable.</t>
         </is>
       </c>
     </row>
@@ -510,7 +509,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Successful login using valid credentials with SIGN IN button</t>
+          <t>Login with valid username and password</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -526,15 +525,15 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Open the login page URL
-Enter haklarr in the User Name field
-Enter Icstunnel1 in the Password field
-Click the SIGN IN button</t>
+          <t>Navigate to the login page URL
+Enter hacklarr in username_textbox
+Enter Icstunnel1 in password_textbox
+Click sign_in_button</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>User authentication succeeds and browser navigates to http://172.21.166.115/washtabui/home. The home page content is displayed and the login page is no longer visible.</t>
+          <t>User authentication succeeds and the application redirects to http://172.21.166.115/washtabui/home with the home page fully loaded and the login page no longer visible.</t>
         </is>
       </c>
     </row>
@@ -546,12 +545,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Successful login using Enter key from password field</t>
+          <t>Login with invalid username and valid password</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -562,15 +561,15 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Open the login page URL
-Enter haklarr in the User Name field
-Enter Icstunnel1 in the Password field
-Press Enter while focus is inside the Password field</t>
+          <t>Navigate to the login page URL
+Enter invaliduser in username_textbox
+Enter Icstunnel1 in password_textbox
+Click sign_in_button</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>User authentication succeeds and the browser redirects to http://172.21.166.115/washtabui/home with the home page interface visible.</t>
+          <t>Authentication fails, the user remains on the login page, the browser URL does not change to the home page URL, and a visible login failure message such as 'Sign in failed' or equivalent authentication error is displayed.</t>
         </is>
       </c>
     </row>
@@ -582,7 +581,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Login fails with incorrect password</t>
+          <t>Login with valid username and invalid password</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -598,15 +597,15 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Open the login page URL
-Enter haklarr in the User Name field
-Enter WrongPassword123 in the Password field
-Click the SIGN IN button</t>
+          <t>Navigate to the login page URL
+Enter hacklarr in username_textbox
+Enter wrongpassword in password_textbox
+Click sign_in_button</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Authentication is rejected. A visible login failure message indicating incorrect username or password appears and the browser remains on the login page URL.</t>
+          <t>Authentication fails, the login page remains displayed, the URL does not change to the home page URL, and a visible authentication failure message is shown.</t>
         </is>
       </c>
     </row>
@@ -618,7 +617,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Login fails with incorrect username</t>
+          <t>Attempt login with empty username and password</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -634,15 +633,15 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Open the login page URL
-Enter wronguser in the User Name field
-Enter Icstunnel1 in the Password field
-Click the SIGN IN button</t>
+          <t>Navigate to the login page URL
+Leave username_textbox empty
+Leave password_textbox empty
+Click sign_in_button</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Authentication fails and an observable error message indicating invalid username or password is displayed while the browser remains on the login page.</t>
+          <t>Login is rejected, the user remains on the login page, the home page URL is not loaded, and the form displays a validation or authentication error preventing login.</t>
         </is>
       </c>
     </row>
@@ -654,7 +653,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Login fails when both username and password are blank</t>
+          <t>Attempt login with valid username and empty password</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -670,15 +669,15 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Open the login page URL
-Leave User Name field empty
-Leave Password field empty
-Click the SIGN IN button</t>
+          <t>Navigate to the login page URL
+Enter hacklarr in username_textbox
+Leave password_textbox empty
+Click sign_in_button</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Login is blocked. Required field validation indicators appear for both User Name and Password fields and the browser remains on the login page.</t>
+          <t>Authentication fails, the application remains on the login page without redirecting to the home page URL, and a visible validation or login error is displayed.</t>
         </is>
       </c>
     </row>
@@ -690,12 +689,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Login fails when username is blank</t>
+          <t>Verify password field masks entered characters</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -706,15 +705,15 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Open the login page URL
-Leave User Name field empty
-Enter Icstunnel1 in the Password field
-Click the SIGN IN button</t>
+          <t>Navigate to the login page URL
+Click password_textbox
+Enter Icstunnel1 in password_textbox
+Observe how characters are displayed</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Submission is rejected with a visible validation message indicating User Name is required and the page remains on the login screen.</t>
+          <t>Characters entered into password_textbox are displayed as masked symbols (such as dots or asterisks) and the actual password text is not visible on screen.</t>
         </is>
       </c>
     </row>
@@ -726,12 +725,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Login fails when password is blank</t>
+          <t>Verify back navigation button redirects to home page</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -742,15 +741,13 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Open the login page URL
-Enter haklarr in the User Name field
-Leave Password field empty
-Click the SIGN IN button</t>
+          <t>Navigate to the login page URL
+Click back_navigation_button</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Submission is rejected with a visible validation message indicating Password is required and the login page remains displayed.</t>
+          <t>Application navigates away from the login page and loads the home page with the browser URL changing to http://172.21.166.115/washtabui/home.</t>
         </is>
       </c>
     </row>
@@ -762,7 +759,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Password field masks entered characters</t>
+          <t>Verify home navigation button redirects to home page</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -778,14 +775,13 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Open the login page URL
-Click inside the Password field
-Type Icstunnel1</t>
+          <t>Navigate to the login page URL
+Click home_navigation_button</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Each typed character in the Password field appears as a masked symbol such as dots or asterisks instead of displaying the actual characters.</t>
+          <t>Application redirects to the home page and the browser URL becomes http://172.21.166.115/washtabui/home with the login page no longer displayed.</t>
         </is>
       </c>
     </row>
@@ -797,12 +793,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Navigation using Home control from login page</t>
+          <t>Login attempt with leading and trailing whitespace in username</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -813,13 +809,15 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Open the login page URL
-Click the Home control</t>
+          <t>Navigate to the login page URL
+Enter '  hacklarr  ' in username_textbox including spaces before and after the username
+Enter Icstunnel1 in password_textbox
+Click sign_in_button</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Browser navigates to http://172.21.166.115/washtabui/home and the home page UI becomes visible.</t>
+          <t>System processes the entered value and rejects authentication, the user remains on the login page, the URL does not change to the home page URL, and a login failure message is displayed.</t>
         </is>
       </c>
     </row>
@@ -831,12 +829,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Navigation using Arrow Back control from login page</t>
+          <t>Login with very long username value</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -847,13 +845,15 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Open the login page URL
-Click the Arrow Back control</t>
+          <t>Navigate to the login page URL
+Enter a username string significantly longer than a typical username length in username_textbox
+Enter Icstunnel1 in password_textbox
+Click sign_in_button</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Browser redirects to http://172.21.166.115/washtabui/home and the home page content loads successfully.</t>
+          <t>Application safely rejects the authentication attempt, the login page remains displayed, no navigation to the home page occurs, and the UI remains stable without page crash or layout break.</t>
         </is>
       </c>
     </row>
@@ -865,7 +865,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Login with leading and trailing spaces in username</t>
+          <t>Login with special characters in username</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -881,15 +881,15 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Open the login page URL
-Enter '  haklarr  ' in the User Name field including leading and trailing spaces
-Enter Icstunnel1 in the Password field
-Click the SIGN IN button</t>
+          <t>Navigate to the login page URL
+Enter user!@# in username_textbox
+Enter Icstunnel1 in password_textbox
+Click sign_in_button</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>System trims leading and trailing spaces from the username before authentication and successfully redirects the user to http://172.21.166.115/washtabui/home.</t>
+          <t>Authentication fails, the user stays on the login page, the home page URL is not loaded, and an authentication failure message is displayed.</t>
         </is>
       </c>
     </row>
@@ -901,12 +901,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Login attempt with whitespace-only username</t>
+          <t>Rapid multiple clicks on SIGN IN button with valid credentials</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -917,195 +917,15 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Open the login page URL
-Enter multiple spaces in the User Name field
-Enter Icstunnel1 in the Password field
-Click the SIGN IN button</t>
+          <t>Navigate to the login page URL
+Enter hacklarr in username_textbox
+Enter Icstunnel1 in password_textbox
+Rapidly click sign_in_button multiple times</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>System treats the username as empty and displays a required-field validation for User Name while remaining on the login page.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>WT-LOGIN14</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Login attempt with whitespace-only password</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Open the login page URL
-Enter haklarr in the User Name field
-Enter multiple spaces in the Password field
-Click the SIGN IN button</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Authentication is rejected and a validation or login failure message appears while the browser remains on the login page.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>WT-LOGIN15</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Login attempt with excessively long username input</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Edge</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Open the login page URL
-Enter a username string longer than 200 characters in the User Name field
-Enter Icstunnel1 in the Password field
-Click the SIGN IN button</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Application does not crash or break UI layout. Authentication fails and an error message is shown while the user remains on the login page.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>WT-LOGIN16</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Login attempt with special characters in username</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Edge</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Open the login page URL
-Enter user!@# in the User Name field
-Enter Icstunnel1 in the Password field
-Click the SIGN IN button</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>Authentication fails and a visible login error message appears while the page remains on the login screen.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>WT-LOGIN17</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Repeated clicking of SIGN IN button during login attempt</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Edge</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Open the login page URL
-Enter haklarr in the User Name field
-Enter Icstunnel1 in the Password field
-Rapidly click the SIGN IN button multiple times</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Only one authentication process is executed and the browser performs a single redirect to http://172.21.166.115/washtabui/home without duplicate navigation or UI errors.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>WT-LOGIN18</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Login attempt with correct username but wrong case password</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Open the login page URL
-Enter haklarr in the User Name field
-Enter icstunnel1 in the Password field
-Click the SIGN IN button</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Authentication fails due to password case sensitivity. An invalid credential message appears and the browser remains on the login page.</t>
+          <t>System processes only one authentication request and redirects a single time to http://172.21.166.115/washtabui/home without duplicate navigation, duplicate sessions, or UI errors.</t>
         </is>
       </c>
     </row>

</xml_diff>